<commit_message>
Feature: enviament d'email real i detecció d'idioma robusta
</commit_message>
<xml_diff>
--- a/tmp/lasecre_34640291370_T2-2026_20260402.xlsx
+++ b/tmp/lasecre_34640291370_T2-2026_20260402.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>Data Registre</t>
   </si>
@@ -61,15 +61,12 @@
     <t>Restauració</t>
   </si>
   <si>
-    <t>https://v5.airtableusercontent.com/v3/u/51/51/1775131200000/OujEJuk5IGQ3M3NNsGzL7g/Q4cHXChdwMRa9LEoEsaFq-x28Uw22TSVQ0HdfMU82epKsXHEvODsGPzMhn-GHpedkIj8nYW3O6Sx1vO8JHtt2nT46ZKxrp33iA4yvSLbkwvcFgM-hG3MgQZS-5fSUza-tc57Re_GAOnDNVnbjwX7vA/1xbbmuXk-m7xllRoyP2wawZWz14kS9qWSPGIjYHt_6c</t>
+    <t>🔗 Veure tiquet</t>
   </si>
   <si>
     <t>1/4/2026 17:23:28</t>
   </si>
   <si>
-    <t>https://v5.airtableusercontent.com/v3/u/51/51/1775131200000/6alDTdlcKi6Lbs9nM2fBWA/KrprNuW-jo9WWIVG3l63hNRjiHryn-gY3freD2d5EEr1vpAHTXVmtrZ9-9hUwBObxQU3DhePhqh5Y5xlauF0maiR-Qx4amkNb89jUNe0EinjoewvLLvXYDQ3mXa5ME0srVPJUKpFbEUEoZVlQ4EoTA/BzdPlbUygBKrl3isaHtiB-xbDyPbNHLcYLzkAIfp-f0</t>
-  </si>
-  <si>
     <t>1/4/2026 17:28:45</t>
   </si>
   <si>
@@ -79,9 +76,6 @@
     <t>Restaurante</t>
   </si>
   <si>
-    <t>https://v5.airtableusercontent.com/v3/u/51/51/1775131200000/7SunoTnRqe7QRCFzU2z2hA/tTKMVlgEs0wQJeU6wpGlilq-9G0ITnveqJ1YQFHVE_v14lDyr9mu-RLp5k1B4YLBuY81wnhDcS9yHn366cz3YGz4Q5_4lxX3pY-_XiwOQjQBLUF8YYaKItfEvQ4VKN565okGW_73WrGrwQzRWy4NQA/BzuvX62bfIFE4pwkFdEj48PAB47kdbdWdjWYSPu2yKE</t>
-  </si>
-  <si>
     <t>1/4/2026 17:50:31</t>
   </si>
   <si>
@@ -100,13 +94,7 @@
     <t>Restauración</t>
   </si>
   <si>
-    <t>https://v5.airtableusercontent.com/v3/u/51/51/1775131200000/T9W4h0hqturOUQ2HyAaCbQ/K_NrDEJqSdjyH0LkDBqwOFEg6MkG5SLFvxmMHERKmvwyg_04m_So-YQUEmLMyGvf953Ta207JKFOWAg9QtB-JSqWvXpQqknwUN7dvNTznLV3fkUDEZ4fiFyIwMx29J8QGCVswObsExSupay-9zAggQ/ORwRlyaGl707kxpD0ESpUg5Bacj5HRf9HF_nBK8T0Ro</t>
-  </si>
-  <si>
     <t>2/4/2026 9:48:11</t>
-  </si>
-  <si>
-    <t>https://v5.airtableusercontent.com/v3/u/51/51/1775131200000/3vGgh8WX3_WrMFVY5LLPPg/gPZAdpwA3vkc8RCI1JGBfa6DqRpvhLB8ehOpTJ_XeAZtAO6p9N1UDAj7_gAIofWNP9n43KEgEdLHeNPqDhREIRn7IdtlH9J__Cpw-alG_O6eM_u1JqvWynnpcIkzNGnrpEhKQOeUNkT2okeP8oKOwA/QT89Qkt8jushAiRoMxOR-N39GOwEA9_LZQg7BQ0pYKk</t>
   </si>
 </sst>
 </file>
@@ -594,18 +582,18 @@
         <v>15</v>
       </c>
       <c r="L3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G4">
         <v>94.7</v>
@@ -620,30 +608,30 @@
         <v>8.61</v>
       </c>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L4" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
       </c>
       <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
+      <c r="F5" t="s">
         <v>25</v>
-      </c>
-      <c r="E5" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>27</v>
       </c>
       <c r="G5">
         <v>94.7</v>
@@ -658,30 +646,30 @@
         <v>8.61</v>
       </c>
       <c r="K5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>27</v>
       </c>
       <c r="G6">
         <v>94.7</v>
@@ -696,13 +684,20 @@
         <v>8.61</v>
       </c>
       <c r="K6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L6" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L2" r:id="rId1" tooltip="Obrir imatge"/>
+    <hyperlink ref="L3" r:id="rId2" tooltip="Obrir imatge"/>
+    <hyperlink ref="L4" r:id="rId3" tooltip="Obrir imatge"/>
+    <hyperlink ref="L5" r:id="rId4" tooltip="Obrir imatge"/>
+    <hyperlink ref="L6" r:id="rId5" tooltip="Obrir imatge"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>